<commit_message>
Major update of statistical analyses for resubmission dec 2025, removed scRNAseq folder
</commit_message>
<xml_diff>
--- a/OtherAnalyses/SKOV3/data/Survival.xlsx
+++ b/OtherAnalyses/SKOV3/data/Survival.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24B74207-7015-4FE0-A485-AFD971C0ED16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D0AAA1A-69A7-46E5-9E23-6CA95AB3F88E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14415" yWindow="-16200" windowWidth="14385" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -430,15 +430,15 @@
   <cols>
     <col min="1" max="1" width="11.28515625" customWidth="1"/>
     <col min="2" max="2" width="6.5703125" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" customWidth="1"/>
-    <col min="4" max="4" width="22.140625" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" customWidth="1"/>
-    <col min="7" max="7" width="16.5703125" customWidth="1"/>
-    <col min="8" max="8" width="15.42578125" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" customWidth="1"/>
-    <col min="10" max="10" width="18.85546875" customWidth="1"/>
-    <col min="11" max="11" width="13.28515625" customWidth="1"/>
+    <col min="3" max="3" width="18.5703125" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="22.140625" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="18.7109375" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="15.42578125" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="20.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -505,10 +505,10 @@
         <v>30</v>
       </c>
       <c r="B3">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -525,10 +525,10 @@
         <v>30</v>
       </c>
       <c r="B4">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
@@ -545,10 +545,10 @@
         <v>30</v>
       </c>
       <c r="B5">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -565,19 +565,19 @@
         <v>30</v>
       </c>
       <c r="B6">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D6" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E6">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F6">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -585,19 +585,19 @@
         <v>30</v>
       </c>
       <c r="B7">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F7">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -605,19 +605,19 @@
         <v>30</v>
       </c>
       <c r="B8">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
       </c>
       <c r="E8">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F8">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -625,19 +625,19 @@
         <v>30</v>
       </c>
       <c r="B9">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E9">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F9">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -645,19 +645,19 @@
         <v>30</v>
       </c>
       <c r="B10">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E10">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F10">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
@@ -665,19 +665,19 @@
         <v>30</v>
       </c>
       <c r="B11">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D11" t="s">
         <v>8</v>
       </c>
       <c r="E11">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F11">
-        <v>31</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -685,22 +685,19 @@
         <v>30</v>
       </c>
       <c r="B12">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
         <v>7</v>
       </c>
-      <c r="G12" t="s">
-        <v>8</v>
-      </c>
-      <c r="H12">
-        <v>1</v>
-      </c>
-      <c r="I12">
-        <v>116</v>
-      </c>
-      <c r="J12">
-        <v>116</v>
+      <c r="D12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12">
+        <v>31</v>
+      </c>
+      <c r="F12">
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -708,22 +705,19 @@
         <v>30</v>
       </c>
       <c r="B13">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="C13" t="s">
         <v>7</v>
       </c>
-      <c r="G13" t="s">
-        <v>8</v>
-      </c>
-      <c r="H13">
-        <v>1</v>
-      </c>
-      <c r="I13">
-        <v>116</v>
-      </c>
-      <c r="J13">
-        <v>116</v>
+      <c r="D13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13">
+        <v>31</v>
+      </c>
+      <c r="F13">
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -731,22 +725,19 @@
         <v>30</v>
       </c>
       <c r="B14">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="C14" t="s">
         <v>7</v>
       </c>
-      <c r="G14" t="s">
-        <v>8</v>
-      </c>
-      <c r="H14">
-        <v>1</v>
-      </c>
-      <c r="I14">
-        <v>116</v>
-      </c>
-      <c r="J14">
-        <v>116</v>
+      <c r="D14" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14">
+        <v>31</v>
+      </c>
+      <c r="F14">
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -754,22 +745,19 @@
         <v>30</v>
       </c>
       <c r="B15">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="C15" t="s">
         <v>7</v>
       </c>
-      <c r="G15" t="s">
-        <v>8</v>
-      </c>
-      <c r="H15">
-        <v>1</v>
-      </c>
-      <c r="I15">
-        <v>116</v>
-      </c>
-      <c r="J15">
-        <v>116</v>
+      <c r="D15" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15">
+        <v>31</v>
+      </c>
+      <c r="F15">
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -777,22 +765,31 @@
         <v>30</v>
       </c>
       <c r="B16">
-        <v>53</v>
+        <v>22</v>
       </c>
       <c r="C16" t="s">
-        <v>7</v>
+        <v>3</v>
+      </c>
+      <c r="D16" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16">
+        <v>23</v>
+      </c>
+      <c r="F16">
+        <v>23</v>
       </c>
       <c r="G16" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H16">
         <v>1</v>
       </c>
       <c r="I16">
-        <v>116</v>
+        <v>103</v>
       </c>
       <c r="J16">
-        <v>116</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -800,10 +797,19 @@
         <v>30</v>
       </c>
       <c r="B17">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>7</v>
+        <v>3</v>
+      </c>
+      <c r="D17" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17">
+        <v>25</v>
+      </c>
+      <c r="F17">
+        <v>25</v>
       </c>
       <c r="G17" t="s">
         <v>8</v>
@@ -812,10 +818,10 @@
         <v>1</v>
       </c>
       <c r="I17">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J17">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -823,22 +829,19 @@
         <v>30</v>
       </c>
       <c r="B18">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>7</v>
-      </c>
-      <c r="G18" t="s">
-        <v>8</v>
-      </c>
-      <c r="H18">
-        <v>1</v>
-      </c>
-      <c r="I18">
-        <v>116</v>
-      </c>
-      <c r="J18">
-        <v>116</v>
+        <v>3</v>
+      </c>
+      <c r="D18" t="s">
+        <v>9</v>
+      </c>
+      <c r="E18">
+        <v>22</v>
+      </c>
+      <c r="F18">
+        <v>22</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -846,22 +849,19 @@
         <v>30</v>
       </c>
       <c r="B19">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="C19" t="s">
-        <v>7</v>
-      </c>
-      <c r="G19" t="s">
-        <v>8</v>
-      </c>
-      <c r="H19">
-        <v>1</v>
-      </c>
-      <c r="I19">
-        <v>116</v>
-      </c>
-      <c r="J19">
-        <v>116</v>
+        <v>3</v>
+      </c>
+      <c r="D19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19">
+        <v>22</v>
+      </c>
+      <c r="F19">
+        <v>22</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -869,19 +869,31 @@
         <v>30</v>
       </c>
       <c r="B20">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="C20" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D20" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E20">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F20">
-        <v>31</v>
+        <v>22</v>
+      </c>
+      <c r="G20" t="s">
+        <v>8</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+      <c r="I20">
+        <v>115</v>
+      </c>
+      <c r="J20">
+        <v>115</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -889,19 +901,19 @@
         <v>30</v>
       </c>
       <c r="B21">
+        <v>27</v>
+      </c>
+      <c r="C21" t="s">
         <v>3</v>
       </c>
-      <c r="C21" t="s">
-        <v>1</v>
-      </c>
       <c r="D21" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E21">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F21">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -909,19 +921,31 @@
         <v>30</v>
       </c>
       <c r="B22">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="C22" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E22">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F22">
-        <v>31</v>
+        <v>28</v>
+      </c>
+      <c r="G22" t="s">
+        <v>8</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
+      <c r="I22">
+        <v>115</v>
+      </c>
+      <c r="J22">
+        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -929,10 +953,10 @@
         <v>30</v>
       </c>
       <c r="B23">
-        <v>44</v>
+        <v>29</v>
       </c>
       <c r="C23" t="s">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D23" t="s">
         <v>8</v>
@@ -949,19 +973,19 @@
         <v>30</v>
       </c>
       <c r="B24">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C24" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D24" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E24">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="F24">
-        <v>31</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -969,19 +993,19 @@
         <v>30</v>
       </c>
       <c r="B25">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D25" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E25">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="F25">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -989,19 +1013,31 @@
         <v>30</v>
       </c>
       <c r="B26">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C26" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D26" t="s">
         <v>9</v>
       </c>
       <c r="E26">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F26">
-        <v>23</v>
+        <v>25</v>
+      </c>
+      <c r="G26" t="s">
+        <v>13</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26">
+        <v>96</v>
+      </c>
+      <c r="J26">
+        <v>96</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -1009,19 +1045,31 @@
         <v>30</v>
       </c>
       <c r="B27">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="C27" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D27" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E27">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="F27">
-        <v>18</v>
+        <v>28</v>
+      </c>
+      <c r="G27" t="s">
+        <v>8</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+      <c r="I27">
+        <v>115</v>
+      </c>
+      <c r="J27">
+        <v>115</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -1029,10 +1077,10 @@
         <v>30</v>
       </c>
       <c r="B28">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="C28" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D28" t="s">
         <v>9</v>
@@ -1049,31 +1097,19 @@
         <v>30</v>
       </c>
       <c r="B29">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="C29" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D29" t="s">
         <v>9</v>
       </c>
       <c r="E29">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F29">
-        <v>23</v>
-      </c>
-      <c r="G29" t="s">
-        <v>12</v>
-      </c>
-      <c r="H29">
-        <v>1</v>
-      </c>
-      <c r="I29">
-        <v>103</v>
-      </c>
-      <c r="J29">
-        <v>103</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
@@ -1081,31 +1117,31 @@
         <v>30</v>
       </c>
       <c r="B30">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C30" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" t="s">
         <v>9</v>
       </c>
       <c r="E30">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F30">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G30" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H30">
         <v>1</v>
       </c>
       <c r="I30">
-        <v>115</v>
+        <v>99</v>
       </c>
       <c r="J30">
-        <v>115</v>
+        <v>99</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
@@ -1113,10 +1149,10 @@
         <v>30</v>
       </c>
       <c r="B31">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="C31" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D31" t="s">
         <v>9</v>
@@ -1127,25 +1163,49 @@
       <c r="F31">
         <v>22</v>
       </c>
+      <c r="G31" t="s">
+        <v>12</v>
+      </c>
+      <c r="H31">
+        <v>1</v>
+      </c>
+      <c r="I31">
+        <v>94</v>
+      </c>
+      <c r="J31">
+        <v>94</v>
+      </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>30</v>
       </c>
       <c r="B32">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="C32" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D32" t="s">
         <v>9</v>
       </c>
       <c r="E32">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F32">
-        <v>22</v>
+        <v>21</v>
+      </c>
+      <c r="G32" t="s">
+        <v>12</v>
+      </c>
+      <c r="H32">
+        <v>1</v>
+      </c>
+      <c r="I32">
+        <v>108</v>
+      </c>
+      <c r="J32">
+        <v>108</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
@@ -1153,31 +1213,19 @@
         <v>30</v>
       </c>
       <c r="B33">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D33" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E33">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="F33">
-        <v>22</v>
-      </c>
-      <c r="G33" t="s">
-        <v>8</v>
-      </c>
-      <c r="H33">
-        <v>1</v>
-      </c>
-      <c r="I33">
-        <v>115</v>
-      </c>
-      <c r="J33">
-        <v>115</v>
+        <v>31</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
@@ -1185,19 +1233,19 @@
         <v>30</v>
       </c>
       <c r="B34">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="C34" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D34" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E34">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F34">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
@@ -1205,31 +1253,19 @@
         <v>30</v>
       </c>
       <c r="B35">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C35" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E35">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F35">
-        <v>28</v>
-      </c>
-      <c r="G35" t="s">
-        <v>8</v>
-      </c>
-      <c r="H35">
-        <v>1</v>
-      </c>
-      <c r="I35">
-        <v>115</v>
-      </c>
-      <c r="J35">
-        <v>115</v>
+        <v>31</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
@@ -1237,31 +1273,19 @@
         <v>30</v>
       </c>
       <c r="B36">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C36" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D36" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E36">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F36">
-        <v>23</v>
-      </c>
-      <c r="G36" t="s">
-        <v>8</v>
-      </c>
-      <c r="H36">
-        <v>1</v>
-      </c>
-      <c r="I36">
-        <v>115</v>
-      </c>
-      <c r="J36">
-        <v>115</v>
+        <v>31</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -1269,19 +1293,19 @@
         <v>30</v>
       </c>
       <c r="B37">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C37" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D37" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E37">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F37">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
@@ -1289,19 +1313,19 @@
         <v>30</v>
       </c>
       <c r="B38">
-        <v>6</v>
+        <v>45</v>
       </c>
       <c r="C38" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D38" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E38">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="F38">
-        <v>23</v>
+        <v>31</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
@@ -1309,19 +1333,19 @@
         <v>30</v>
       </c>
       <c r="B39">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="C39" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D39" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E39">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="F39">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
@@ -1329,19 +1353,31 @@
         <v>30</v>
       </c>
       <c r="B40">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="C40" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D40" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E40">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F40">
-        <v>10</v>
+        <v>23</v>
+      </c>
+      <c r="G40" t="s">
+        <v>8</v>
+      </c>
+      <c r="H40">
+        <v>1</v>
+      </c>
+      <c r="I40">
+        <v>115</v>
+      </c>
+      <c r="J40">
+        <v>115</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
@@ -1349,19 +1385,19 @@
         <v>30</v>
       </c>
       <c r="B41">
-        <v>30</v>
+        <v>48</v>
       </c>
       <c r="C41" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D41" t="s">
         <v>9</v>
       </c>
       <c r="E41">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F41">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
@@ -1369,19 +1405,22 @@
         <v>30</v>
       </c>
       <c r="B42">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="C42" t="s">
-        <v>4</v>
-      </c>
-      <c r="D42" t="s">
-        <v>9</v>
-      </c>
-      <c r="E42">
-        <v>23</v>
-      </c>
-      <c r="F42">
-        <v>23</v>
+        <v>7</v>
+      </c>
+      <c r="G42" t="s">
+        <v>8</v>
+      </c>
+      <c r="H42">
+        <v>1</v>
+      </c>
+      <c r="I42">
+        <v>116</v>
+      </c>
+      <c r="J42">
+        <v>116</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
@@ -1389,31 +1428,22 @@
         <v>30</v>
       </c>
       <c r="B43">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="C43" t="s">
-        <v>4</v>
-      </c>
-      <c r="D43" t="s">
-        <v>9</v>
-      </c>
-      <c r="E43">
-        <v>25</v>
-      </c>
-      <c r="F43">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G43" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="H43">
         <v>1</v>
       </c>
       <c r="I43">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="J43">
-        <v>96</v>
+        <v>116</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -1421,19 +1451,10 @@
         <v>30</v>
       </c>
       <c r="B44">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="C44" t="s">
-        <v>4</v>
-      </c>
-      <c r="D44" t="s">
-        <v>9</v>
-      </c>
-      <c r="E44">
-        <v>28</v>
-      </c>
-      <c r="F44">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="G44" t="s">
         <v>8</v>
@@ -1442,10 +1463,10 @@
         <v>1</v>
       </c>
       <c r="I44">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="J44">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -1453,19 +1474,22 @@
         <v>30</v>
       </c>
       <c r="B45">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="C45" t="s">
-        <v>4</v>
-      </c>
-      <c r="D45" t="s">
-        <v>9</v>
-      </c>
-      <c r="E45">
-        <v>28</v>
-      </c>
-      <c r="F45">
-        <v>28</v>
+        <v>7</v>
+      </c>
+      <c r="G45" t="s">
+        <v>8</v>
+      </c>
+      <c r="H45">
+        <v>1</v>
+      </c>
+      <c r="I45">
+        <v>116</v>
+      </c>
+      <c r="J45">
+        <v>116</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
@@ -1473,19 +1497,22 @@
         <v>30</v>
       </c>
       <c r="B46">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="C46" t="s">
-        <v>4</v>
-      </c>
-      <c r="D46" t="s">
-        <v>9</v>
-      </c>
-      <c r="E46">
-        <v>22</v>
-      </c>
-      <c r="F46">
-        <v>22</v>
+        <v>7</v>
+      </c>
+      <c r="G46" t="s">
+        <v>8</v>
+      </c>
+      <c r="H46">
+        <v>1</v>
+      </c>
+      <c r="I46">
+        <v>116</v>
+      </c>
+      <c r="J46">
+        <v>116</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
@@ -1493,31 +1520,22 @@
         <v>30</v>
       </c>
       <c r="B47">
-        <v>36</v>
+        <v>54</v>
       </c>
       <c r="C47" t="s">
-        <v>4</v>
-      </c>
-      <c r="D47" t="s">
-        <v>9</v>
-      </c>
-      <c r="E47">
-        <v>23</v>
-      </c>
-      <c r="F47">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="G47" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H47">
         <v>1</v>
       </c>
       <c r="I47">
-        <v>99</v>
+        <v>116</v>
       </c>
       <c r="J47">
-        <v>99</v>
+        <v>116</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
@@ -1525,31 +1543,22 @@
         <v>30</v>
       </c>
       <c r="B48">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="C48" t="s">
-        <v>4</v>
-      </c>
-      <c r="D48" t="s">
-        <v>9</v>
-      </c>
-      <c r="E48">
-        <v>22</v>
-      </c>
-      <c r="F48">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="G48" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H48">
         <v>1</v>
       </c>
       <c r="I48">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="J48">
-        <v>94</v>
+        <v>116</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
@@ -1557,31 +1566,22 @@
         <v>30</v>
       </c>
       <c r="B49">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="C49" t="s">
-        <v>4</v>
-      </c>
-      <c r="D49" t="s">
-        <v>9</v>
-      </c>
-      <c r="E49">
-        <v>21</v>
-      </c>
-      <c r="F49">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="G49" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H49">
         <v>1</v>
       </c>
       <c r="I49">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="J49">
-        <v>108</v>
+        <v>116</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.25">
@@ -1635,22 +1635,37 @@
         <v>32</v>
       </c>
       <c r="B52">
+        <v>3</v>
+      </c>
+      <c r="C52" t="s">
+        <v>5</v>
+      </c>
+      <c r="D52" t="s">
+        <v>10</v>
+      </c>
+      <c r="E52">
+        <v>119</v>
+      </c>
+      <c r="F52">
+        <v>45</v>
+      </c>
+      <c r="G52" t="s">
         <v>13</v>
       </c>
-      <c r="C52" t="s">
-        <v>7</v>
-      </c>
-      <c r="D52" t="s">
-        <v>8</v>
-      </c>
-      <c r="E52">
-        <v>52</v>
-      </c>
-      <c r="F52">
-        <v>52</v>
+      <c r="H52">
+        <v>1</v>
+      </c>
+      <c r="I52">
+        <v>119</v>
+      </c>
+      <c r="J52">
+        <v>114</v>
+      </c>
+      <c r="K52">
+        <v>45</v>
       </c>
       <c r="L52">
-        <v>52</v>
+        <v>119</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.25">
@@ -1658,22 +1673,34 @@
         <v>32</v>
       </c>
       <c r="B53">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C53" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D53" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E53">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="F53">
-        <v>52</v>
+        <v>25</v>
+      </c>
+      <c r="G53" t="s">
+        <v>8</v>
+      </c>
+      <c r="H53">
+        <v>1</v>
+      </c>
+      <c r="I53">
+        <v>119</v>
+      </c>
+      <c r="J53">
+        <v>119</v>
       </c>
       <c r="L53">
-        <v>52</v>
+        <v>119</v>
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.25">
@@ -1681,22 +1708,34 @@
         <v>32</v>
       </c>
       <c r="B54">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C54" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D54" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E54">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="F54">
-        <v>52</v>
+        <v>30</v>
+      </c>
+      <c r="G54" t="s">
+        <v>25</v>
+      </c>
+      <c r="H54">
+        <v>0</v>
+      </c>
+      <c r="I54">
+        <v>92</v>
+      </c>
+      <c r="J54">
+        <v>92</v>
       </c>
       <c r="L54">
-        <v>52</v>
+        <v>119</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.25">
@@ -1704,22 +1743,34 @@
         <v>32</v>
       </c>
       <c r="B55">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="C55" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D55" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E55">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="F55">
-        <v>52</v>
+        <v>25</v>
+      </c>
+      <c r="G55" t="s">
+        <v>8</v>
+      </c>
+      <c r="H55">
+        <v>1</v>
+      </c>
+      <c r="I55">
+        <v>119</v>
+      </c>
+      <c r="J55">
+        <v>119</v>
       </c>
       <c r="L55">
-        <v>52</v>
+        <v>119</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.25">
@@ -1727,22 +1778,34 @@
         <v>32</v>
       </c>
       <c r="B56">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C56" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D56" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E56">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="F56">
-        <v>52</v>
+        <v>28</v>
+      </c>
+      <c r="G56" t="s">
+        <v>25</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56">
+        <v>92</v>
+      </c>
+      <c r="J56">
+        <v>92</v>
       </c>
       <c r="L56">
-        <v>52</v>
+        <v>119</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.25">
@@ -1750,22 +1813,37 @@
         <v>32</v>
       </c>
       <c r="B57">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="C57" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D57" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E57">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="F57">
-        <v>52</v>
+        <v>30</v>
+      </c>
+      <c r="G57" t="s">
+        <v>25</v>
+      </c>
+      <c r="H57">
+        <v>0</v>
+      </c>
+      <c r="I57">
+        <v>92</v>
+      </c>
+      <c r="J57">
+        <v>92</v>
+      </c>
+      <c r="K57">
+        <v>80</v>
       </c>
       <c r="L57">
-        <v>52</v>
+        <v>119</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.25">
@@ -1773,22 +1851,37 @@
         <v>32</v>
       </c>
       <c r="B58">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C58" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D58" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E58">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="F58">
-        <v>52</v>
+        <v>35</v>
+      </c>
+      <c r="G58" t="s">
+        <v>25</v>
+      </c>
+      <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58">
+        <v>92</v>
+      </c>
+      <c r="J58">
+        <v>92</v>
+      </c>
+      <c r="K58">
+        <v>80</v>
       </c>
       <c r="L58">
-        <v>52</v>
+        <v>119</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.25">
@@ -1796,22 +1889,37 @@
         <v>32</v>
       </c>
       <c r="B59">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C59" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D59" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E59">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="F59">
-        <v>52</v>
+        <v>25</v>
+      </c>
+      <c r="G59" t="s">
+        <v>25</v>
+      </c>
+      <c r="H59">
+        <v>0</v>
+      </c>
+      <c r="I59">
+        <v>92</v>
+      </c>
+      <c r="J59">
+        <v>92</v>
+      </c>
+      <c r="K59">
+        <v>87</v>
       </c>
       <c r="L59">
-        <v>52</v>
+        <v>119</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.25">
@@ -1819,22 +1927,37 @@
         <v>32</v>
       </c>
       <c r="B60">
-        <v>29</v>
+        <v>11</v>
       </c>
       <c r="C60" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D60" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E60">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="F60">
-        <v>52</v>
+        <v>28</v>
+      </c>
+      <c r="G60" t="s">
+        <v>13</v>
+      </c>
+      <c r="H60">
+        <v>1</v>
+      </c>
+      <c r="I60">
+        <v>119</v>
+      </c>
+      <c r="J60">
+        <v>105</v>
+      </c>
+      <c r="K60">
+        <v>80</v>
       </c>
       <c r="L60">
-        <v>52</v>
+        <v>119</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.25">
@@ -1842,7 +1965,7 @@
         <v>32</v>
       </c>
       <c r="B61">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="C61" t="s">
         <v>1</v>
@@ -1865,25 +1988,22 @@
         <v>32</v>
       </c>
       <c r="B62">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="C62" t="s">
         <v>7</v>
       </c>
-      <c r="G62" t="s">
-        <v>8</v>
-      </c>
-      <c r="H62">
-        <v>1</v>
-      </c>
-      <c r="I62">
-        <v>119</v>
-      </c>
-      <c r="J62">
-        <v>119</v>
+      <c r="D62" t="s">
+        <v>8</v>
+      </c>
+      <c r="E62">
+        <v>52</v>
+      </c>
+      <c r="F62">
+        <v>52</v>
       </c>
       <c r="L62">
-        <v>119</v>
+        <v>52</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.25">
@@ -1891,25 +2011,22 @@
         <v>32</v>
       </c>
       <c r="B63">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="C63" t="s">
         <v>7</v>
       </c>
-      <c r="G63" t="s">
-        <v>8</v>
-      </c>
-      <c r="H63">
-        <v>1</v>
-      </c>
-      <c r="I63">
-        <v>119</v>
-      </c>
-      <c r="J63">
-        <v>119</v>
+      <c r="D63" t="s">
+        <v>8</v>
+      </c>
+      <c r="E63">
+        <v>52</v>
+      </c>
+      <c r="F63">
+        <v>52</v>
       </c>
       <c r="L63">
-        <v>119</v>
+        <v>52</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
@@ -1917,25 +2034,22 @@
         <v>32</v>
       </c>
       <c r="B64">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="C64" t="s">
         <v>7</v>
       </c>
-      <c r="G64" t="s">
-        <v>8</v>
-      </c>
-      <c r="H64">
-        <v>1</v>
-      </c>
-      <c r="I64">
-        <v>119</v>
-      </c>
-      <c r="J64">
-        <v>119</v>
+      <c r="D64" t="s">
+        <v>8</v>
+      </c>
+      <c r="E64">
+        <v>52</v>
+      </c>
+      <c r="F64">
+        <v>52</v>
       </c>
       <c r="L64">
-        <v>119</v>
+        <v>52</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
@@ -1943,22 +2057,34 @@
         <v>32</v>
       </c>
       <c r="B65">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="C65" t="s">
-        <v>7</v>
+        <v>5</v>
+      </c>
+      <c r="D65" t="s">
+        <v>11</v>
+      </c>
+      <c r="E65">
+        <v>35</v>
+      </c>
+      <c r="F65">
+        <v>35</v>
       </c>
       <c r="G65" t="s">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="H65">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I65">
-        <v>119</v>
+        <v>92</v>
       </c>
       <c r="J65">
-        <v>119</v>
+        <v>92</v>
+      </c>
+      <c r="K65">
+        <v>80</v>
       </c>
       <c r="L65">
         <v>119</v>
@@ -1969,25 +2095,22 @@
         <v>32</v>
       </c>
       <c r="B66">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="C66" t="s">
-        <v>7</v>
-      </c>
-      <c r="G66" t="s">
-        <v>8</v>
-      </c>
-      <c r="H66">
-        <v>1</v>
-      </c>
-      <c r="I66">
-        <v>112</v>
-      </c>
-      <c r="J66">
-        <v>112</v>
+        <v>1</v>
+      </c>
+      <c r="D66" t="s">
+        <v>8</v>
+      </c>
+      <c r="E66">
+        <v>52</v>
+      </c>
+      <c r="F66">
+        <v>52</v>
       </c>
       <c r="L66">
-        <v>119</v>
+        <v>52</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.25">
@@ -1995,25 +2118,22 @@
         <v>32</v>
       </c>
       <c r="B67">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="C67" t="s">
-        <v>7</v>
-      </c>
-      <c r="G67" t="s">
-        <v>8</v>
-      </c>
-      <c r="H67">
-        <v>1</v>
-      </c>
-      <c r="I67">
-        <v>119</v>
-      </c>
-      <c r="J67">
-        <v>119</v>
+        <v>1</v>
+      </c>
+      <c r="D67" t="s">
+        <v>8</v>
+      </c>
+      <c r="E67">
+        <v>52</v>
+      </c>
+      <c r="F67">
+        <v>52</v>
       </c>
       <c r="L67">
-        <v>119</v>
+        <v>52</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.25">
@@ -2021,25 +2141,22 @@
         <v>32</v>
       </c>
       <c r="B68">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="C68" t="s">
-        <v>7</v>
-      </c>
-      <c r="G68" t="s">
-        <v>8</v>
-      </c>
-      <c r="H68">
-        <v>1</v>
-      </c>
-      <c r="I68">
-        <v>119</v>
-      </c>
-      <c r="J68">
-        <v>119</v>
+        <v>1</v>
+      </c>
+      <c r="D68" t="s">
+        <v>8</v>
+      </c>
+      <c r="E68">
+        <v>52</v>
+      </c>
+      <c r="F68">
+        <v>52</v>
       </c>
       <c r="L68">
-        <v>119</v>
+        <v>52</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.25">
@@ -2047,25 +2164,25 @@
         <v>32</v>
       </c>
       <c r="B69">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="C69" t="s">
-        <v>7</v>
-      </c>
-      <c r="G69" t="s">
-        <v>8</v>
-      </c>
-      <c r="H69">
-        <v>1</v>
-      </c>
-      <c r="I69">
-        <v>119</v>
-      </c>
-      <c r="J69">
-        <v>119</v>
+        <v>5</v>
+      </c>
+      <c r="D69" t="s">
+        <v>11</v>
+      </c>
+      <c r="E69">
+        <v>35</v>
+      </c>
+      <c r="F69">
+        <v>35</v>
+      </c>
+      <c r="K69">
+        <v>45</v>
       </c>
       <c r="L69">
-        <v>119</v>
+        <v>80</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.25">
@@ -2073,25 +2190,22 @@
         <v>32</v>
       </c>
       <c r="B70">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="C70" t="s">
-        <v>7</v>
-      </c>
-      <c r="G70" t="s">
-        <v>8</v>
-      </c>
-      <c r="H70">
-        <v>1</v>
-      </c>
-      <c r="I70">
-        <v>119</v>
-      </c>
-      <c r="J70">
-        <v>119</v>
+        <v>5</v>
+      </c>
+      <c r="D70" t="s">
+        <v>8</v>
+      </c>
+      <c r="E70">
+        <v>72</v>
+      </c>
+      <c r="F70">
+        <v>72</v>
       </c>
       <c r="L70">
-        <v>119</v>
+        <v>72</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.25">
@@ -2099,10 +2213,19 @@
         <v>32</v>
       </c>
       <c r="B71">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C71" t="s">
-        <v>7</v>
+        <v>5</v>
+      </c>
+      <c r="D71" t="s">
+        <v>10</v>
+      </c>
+      <c r="E71">
+        <v>119</v>
+      </c>
+      <c r="F71">
+        <v>52</v>
       </c>
       <c r="G71" t="s">
         <v>8</v>
@@ -2115,6 +2238,9 @@
       </c>
       <c r="J71">
         <v>119</v>
+      </c>
+      <c r="K71">
+        <v>87</v>
       </c>
       <c r="L71">
         <v>119</v>
@@ -2125,19 +2251,19 @@
         <v>32</v>
       </c>
       <c r="B72">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="C72" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D72" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E72">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="F72">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G72" t="s">
         <v>8</v>
@@ -2150,6 +2276,9 @@
       </c>
       <c r="J72">
         <v>119</v>
+      </c>
+      <c r="K72">
+        <v>52</v>
       </c>
       <c r="L72">
         <v>119</v>
@@ -2160,19 +2289,19 @@
         <v>32</v>
       </c>
       <c r="B73">
+        <v>24</v>
+      </c>
+      <c r="C73" t="s">
         <v>5</v>
       </c>
-      <c r="C73" t="s">
-        <v>3</v>
-      </c>
       <c r="D73" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E73">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="F73">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="G73" t="s">
         <v>25</v>
@@ -2186,6 +2315,9 @@
       <c r="J73">
         <v>92</v>
       </c>
+      <c r="K73">
+        <v>80</v>
+      </c>
       <c r="L73">
         <v>119</v>
       </c>
@@ -2302,37 +2434,22 @@
         <v>32</v>
       </c>
       <c r="B78">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C78" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D78" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E78">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="F78">
-        <v>28</v>
-      </c>
-      <c r="G78" t="s">
-        <v>8</v>
-      </c>
-      <c r="H78">
-        <v>1</v>
-      </c>
-      <c r="I78">
-        <v>119</v>
-      </c>
-      <c r="J78">
-        <v>119</v>
-      </c>
-      <c r="K78">
-        <v>80</v>
+        <v>52</v>
       </c>
       <c r="L78">
-        <v>119</v>
+        <v>52</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.25">
@@ -2340,37 +2457,22 @@
         <v>32</v>
       </c>
       <c r="B79">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C79" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D79" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E79">
-        <v>30</v>
+        <v>52</v>
       </c>
       <c r="F79">
-        <v>30</v>
-      </c>
-      <c r="G79" t="s">
-        <v>25</v>
-      </c>
-      <c r="H79">
-        <v>0</v>
-      </c>
-      <c r="I79">
-        <v>92</v>
-      </c>
-      <c r="J79">
-        <v>92</v>
-      </c>
-      <c r="K79">
-        <v>87</v>
+        <v>52</v>
       </c>
       <c r="L79">
-        <v>119</v>
+        <v>52</v>
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.25">
@@ -2378,22 +2480,37 @@
         <v>32</v>
       </c>
       <c r="B80">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C80" t="s">
         <v>3</v>
       </c>
       <c r="D80" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E80">
+        <v>28</v>
+      </c>
+      <c r="F80">
+        <v>28</v>
+      </c>
+      <c r="G80" t="s">
+        <v>8</v>
+      </c>
+      <c r="H80">
+        <v>1</v>
+      </c>
+      <c r="I80">
+        <v>119</v>
+      </c>
+      <c r="J80">
+        <v>119</v>
+      </c>
+      <c r="K80">
         <v>80</v>
       </c>
-      <c r="F80">
-        <v>80</v>
-      </c>
       <c r="L80">
-        <v>80</v>
+        <v>119</v>
       </c>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.25">
@@ -2401,34 +2518,34 @@
         <v>32</v>
       </c>
       <c r="B81">
+        <v>32</v>
+      </c>
+      <c r="C81" t="s">
         <v>3</v>
       </c>
-      <c r="C81" t="s">
-        <v>5</v>
-      </c>
       <c r="D81" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E81">
-        <v>119</v>
+        <v>30</v>
       </c>
       <c r="F81">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="G81" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="H81">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I81">
-        <v>119</v>
+        <v>92</v>
       </c>
       <c r="J81">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="K81">
-        <v>45</v>
+        <v>87</v>
       </c>
       <c r="L81">
         <v>119</v>
@@ -2439,34 +2556,31 @@
         <v>32</v>
       </c>
       <c r="B82">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="C82" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D82" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E82">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="F82">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="G82" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="H82">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I82">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="J82">
-        <v>92</v>
-      </c>
-      <c r="K82">
-        <v>80</v>
+        <v>101</v>
       </c>
       <c r="L82">
         <v>119</v>
@@ -2477,25 +2591,37 @@
         <v>32</v>
       </c>
       <c r="B83">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="C83" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D83" t="s">
         <v>11</v>
       </c>
       <c r="E83">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="F83">
-        <v>35</v>
+        <v>25</v>
+      </c>
+      <c r="G83" t="s">
+        <v>25</v>
+      </c>
+      <c r="H83">
+        <v>0</v>
+      </c>
+      <c r="I83">
+        <v>92</v>
+      </c>
+      <c r="J83">
+        <v>92</v>
       </c>
       <c r="K83">
-        <v>45</v>
+        <v>87</v>
       </c>
       <c r="L83">
-        <v>80</v>
+        <v>119</v>
       </c>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.25">
@@ -2503,22 +2629,37 @@
         <v>32</v>
       </c>
       <c r="B84">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="C84" t="s">
         <v>5</v>
       </c>
       <c r="D84" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E84">
-        <v>72</v>
+        <v>119</v>
       </c>
       <c r="F84">
-        <v>72</v>
+        <v>49</v>
+      </c>
+      <c r="G84" t="s">
+        <v>25</v>
+      </c>
+      <c r="H84">
+        <v>0</v>
+      </c>
+      <c r="I84">
+        <v>92</v>
+      </c>
+      <c r="J84">
+        <v>92</v>
+      </c>
+      <c r="K84">
+        <v>87</v>
       </c>
       <c r="L84">
-        <v>72</v>
+        <v>119</v>
       </c>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.25">
@@ -2526,19 +2667,10 @@
         <v>32</v>
       </c>
       <c r="B85">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="C85" t="s">
-        <v>5</v>
-      </c>
-      <c r="D85" t="s">
-        <v>10</v>
-      </c>
-      <c r="E85">
-        <v>119</v>
-      </c>
-      <c r="F85">
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="G85" t="s">
         <v>8</v>
@@ -2551,9 +2683,6 @@
       </c>
       <c r="J85">
         <v>119</v>
-      </c>
-      <c r="K85">
-        <v>87</v>
       </c>
       <c r="L85">
         <v>119</v>
@@ -2564,34 +2693,31 @@
         <v>32</v>
       </c>
       <c r="B86">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="C86" t="s">
         <v>5</v>
       </c>
       <c r="D86" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E86">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="F86">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="G86" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H86">
         <v>1</v>
       </c>
       <c r="I86">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="J86">
-        <v>119</v>
-      </c>
-      <c r="K86">
-        <v>52</v>
+        <v>105</v>
       </c>
       <c r="L86">
         <v>119</v>
@@ -2602,37 +2728,22 @@
         <v>32</v>
       </c>
       <c r="B87">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="C87" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D87" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E87">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="F87">
-        <v>21</v>
-      </c>
-      <c r="G87" t="s">
-        <v>25</v>
-      </c>
-      <c r="H87">
-        <v>0</v>
-      </c>
-      <c r="I87">
-        <v>92</v>
-      </c>
-      <c r="J87">
-        <v>92</v>
-      </c>
-      <c r="K87">
         <v>80</v>
       </c>
       <c r="L87">
-        <v>119</v>
+        <v>80</v>
       </c>
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.25">
@@ -2640,34 +2751,34 @@
         <v>32</v>
       </c>
       <c r="B88">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C88" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D88" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E88">
-        <v>119</v>
+        <v>28</v>
       </c>
       <c r="F88">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="G88" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="H88">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I88">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="J88">
-        <v>92</v>
+        <v>114</v>
       </c>
       <c r="K88">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="L88">
         <v>119</v>
@@ -2678,31 +2789,22 @@
         <v>32</v>
       </c>
       <c r="B89">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C89" t="s">
-        <v>5</v>
-      </c>
-      <c r="D89" t="s">
-        <v>9</v>
-      </c>
-      <c r="E89">
-        <v>21</v>
-      </c>
-      <c r="F89">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="G89" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H89">
         <v>1</v>
       </c>
       <c r="I89">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="J89">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="L89">
         <v>119</v>
@@ -2713,19 +2815,10 @@
         <v>32</v>
       </c>
       <c r="B90">
-        <v>6</v>
+        <v>42</v>
       </c>
       <c r="C90" t="s">
-        <v>4</v>
-      </c>
-      <c r="D90" t="s">
-        <v>9</v>
-      </c>
-      <c r="E90">
-        <v>25</v>
-      </c>
-      <c r="F90">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G90" t="s">
         <v>8</v>
@@ -2748,34 +2841,22 @@
         <v>32</v>
       </c>
       <c r="B91">
+        <v>43</v>
+      </c>
+      <c r="C91" t="s">
         <v>7</v>
       </c>
-      <c r="C91" t="s">
-        <v>4</v>
-      </c>
       <c r="D91" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E91">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="F91">
-        <v>28</v>
-      </c>
-      <c r="G91" t="s">
-        <v>25</v>
-      </c>
-      <c r="H91">
-        <v>0</v>
-      </c>
-      <c r="I91">
-        <v>92</v>
-      </c>
-      <c r="J91">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="L91">
-        <v>119</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.25">
@@ -2783,34 +2864,22 @@
         <v>32</v>
       </c>
       <c r="B92">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="C92" t="s">
-        <v>4</v>
-      </c>
-      <c r="D92" t="s">
-        <v>11</v>
-      </c>
-      <c r="E92">
-        <v>30</v>
-      </c>
-      <c r="F92">
-        <v>30</v>
+        <v>7</v>
       </c>
       <c r="G92" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="H92">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I92">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="J92">
-        <v>92</v>
-      </c>
-      <c r="K92">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="L92">
         <v>119</v>
@@ -2821,34 +2890,22 @@
         <v>32</v>
       </c>
       <c r="B93">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="C93" t="s">
-        <v>4</v>
-      </c>
-      <c r="D93" t="s">
-        <v>11</v>
-      </c>
-      <c r="E93">
-        <v>35</v>
-      </c>
-      <c r="F93">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="G93" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="H93">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I93">
-        <v>92</v>
+        <v>112</v>
       </c>
       <c r="J93">
-        <v>92</v>
-      </c>
-      <c r="K93">
-        <v>80</v>
+        <v>112</v>
       </c>
       <c r="L93">
         <v>119</v>
@@ -2859,34 +2916,22 @@
         <v>32</v>
       </c>
       <c r="B94">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="C94" t="s">
-        <v>4</v>
-      </c>
-      <c r="D94" t="s">
-        <v>11</v>
-      </c>
-      <c r="E94">
-        <v>25</v>
-      </c>
-      <c r="F94">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G94" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="H94">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I94">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="J94">
-        <v>92</v>
-      </c>
-      <c r="K94">
-        <v>87</v>
+        <v>119</v>
       </c>
       <c r="L94">
         <v>119</v>
@@ -2897,22 +2942,13 @@
         <v>32</v>
       </c>
       <c r="B95">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="C95" t="s">
-        <v>4</v>
-      </c>
-      <c r="D95" t="s">
-        <v>11</v>
-      </c>
-      <c r="E95">
-        <v>28</v>
-      </c>
-      <c r="F95">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="G95" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="H95">
         <v>1</v>
@@ -2921,10 +2957,7 @@
         <v>119</v>
       </c>
       <c r="J95">
-        <v>105</v>
-      </c>
-      <c r="K95">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="L95">
         <v>119</v>
@@ -2935,22 +2968,13 @@
         <v>32</v>
       </c>
       <c r="B96">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="C96" t="s">
-        <v>4</v>
-      </c>
-      <c r="D96" t="s">
-        <v>9</v>
-      </c>
-      <c r="E96">
-        <v>25</v>
-      </c>
-      <c r="F96">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G96" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="H96">
         <v>1</v>
@@ -2959,7 +2983,7 @@
         <v>119</v>
       </c>
       <c r="J96">
-        <v>101</v>
+        <v>119</v>
       </c>
       <c r="L96">
         <v>119</v>
@@ -2970,34 +2994,22 @@
         <v>32</v>
       </c>
       <c r="B97">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="C97" t="s">
-        <v>4</v>
-      </c>
-      <c r="D97" t="s">
-        <v>11</v>
-      </c>
-      <c r="E97">
-        <v>25</v>
-      </c>
-      <c r="F97">
-        <v>25</v>
+        <v>7</v>
       </c>
       <c r="G97" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="H97">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I97">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="J97">
-        <v>92</v>
-      </c>
-      <c r="K97">
-        <v>87</v>
+        <v>119</v>
       </c>
       <c r="L97">
         <v>119</v>
@@ -3008,34 +3020,22 @@
         <v>32</v>
       </c>
       <c r="B98">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="C98" t="s">
-        <v>4</v>
-      </c>
-      <c r="D98" t="s">
-        <v>11</v>
-      </c>
-      <c r="E98">
-        <v>28</v>
-      </c>
-      <c r="F98">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="G98" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H98">
         <v>1</v>
       </c>
       <c r="I98">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="J98">
-        <v>114</v>
-      </c>
-      <c r="K98">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="L98">
         <v>119</v>
@@ -3046,19 +3046,37 @@
         <v>43</v>
       </c>
       <c r="B99">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="C99" t="s">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="D99" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E99">
-        <v>72</v>
+        <v>119</v>
+      </c>
+      <c r="F99">
+        <v>24</v>
+      </c>
+      <c r="G99" t="s">
+        <v>25</v>
+      </c>
+      <c r="H99">
+        <v>0</v>
+      </c>
+      <c r="I99">
+        <v>95</v>
+      </c>
+      <c r="J99">
+        <v>95</v>
+      </c>
+      <c r="K99">
+        <v>84</v>
       </c>
       <c r="L99">
-        <v>72</v>
+        <v>119</v>
       </c>
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.25">
@@ -3066,19 +3084,25 @@
         <v>43</v>
       </c>
       <c r="B100">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="C100" t="s">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="D100" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E100">
-        <v>65</v>
+        <v>77</v>
+      </c>
+      <c r="F100">
+        <v>16</v>
+      </c>
+      <c r="K100">
+        <v>21</v>
       </c>
       <c r="L100">
-        <v>65</v>
+        <v>77</v>
       </c>
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.25">
@@ -3086,19 +3110,25 @@
         <v>43</v>
       </c>
       <c r="B101">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="C101" t="s">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="D101" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E101">
-        <v>72</v>
+        <v>92</v>
+      </c>
+      <c r="F101">
+        <v>21</v>
+      </c>
+      <c r="K101">
+        <v>52</v>
       </c>
       <c r="L101">
-        <v>72</v>
+        <v>92</v>
       </c>
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.25">
@@ -3106,19 +3136,25 @@
         <v>43</v>
       </c>
       <c r="B102">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="C102" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="D102" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E102">
-        <v>52</v>
+        <v>95</v>
+      </c>
+      <c r="F102">
+        <v>14</v>
+      </c>
+      <c r="K102">
+        <v>58</v>
       </c>
       <c r="L102">
-        <v>52</v>
+        <v>95</v>
       </c>
     </row>
     <row r="103" spans="1:12" x14ac:dyDescent="0.25">
@@ -3126,10 +3162,10 @@
         <v>43</v>
       </c>
       <c r="B103">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="C103" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="D103" t="s">
         <v>8</v>
@@ -3146,19 +3182,37 @@
         <v>43</v>
       </c>
       <c r="B104">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="C104" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="D104" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E104">
+        <v>35</v>
+      </c>
+      <c r="F104">
+        <v>35</v>
+      </c>
+      <c r="G104" t="s">
+        <v>12</v>
+      </c>
+      <c r="H104">
+        <v>1</v>
+      </c>
+      <c r="I104">
+        <v>112</v>
+      </c>
+      <c r="J104">
+        <v>112</v>
+      </c>
+      <c r="K104">
         <v>77</v>
       </c>
       <c r="L104">
-        <v>77</v>
+        <v>119</v>
       </c>
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.25">
@@ -3166,7 +3220,7 @@
         <v>43</v>
       </c>
       <c r="B105">
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="C105" t="s">
         <v>22</v>
@@ -3186,37 +3240,19 @@
         <v>43</v>
       </c>
       <c r="B106">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="C106" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="D106" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E106">
-        <v>119</v>
-      </c>
-      <c r="F106">
-        <v>24</v>
-      </c>
-      <c r="G106" t="s">
-        <v>25</v>
-      </c>
-      <c r="H106">
-        <v>0</v>
-      </c>
-      <c r="I106">
-        <v>95</v>
-      </c>
-      <c r="J106">
-        <v>95</v>
-      </c>
-      <c r="K106">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="L106">
-        <v>119</v>
+        <v>65</v>
       </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.25">
@@ -3224,25 +3260,19 @@
         <v>43</v>
       </c>
       <c r="B107">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="C107" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="D107" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E107">
-        <v>77</v>
-      </c>
-      <c r="F107">
-        <v>16</v>
-      </c>
-      <c r="K107">
-        <v>21</v>
+        <v>72</v>
       </c>
       <c r="L107">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.25">
@@ -3250,25 +3280,19 @@
         <v>43</v>
       </c>
       <c r="B108">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="C108" t="s">
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="D108" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E108">
-        <v>92</v>
-      </c>
-      <c r="F108">
-        <v>21</v>
-      </c>
-      <c r="K108">
         <v>52</v>
       </c>
       <c r="L108">
-        <v>92</v>
+        <v>52</v>
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.25">
@@ -3316,25 +3340,37 @@
         <v>43</v>
       </c>
       <c r="B111">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C111" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D111" t="s">
         <v>10</v>
       </c>
       <c r="E111">
+        <v>119</v>
+      </c>
+      <c r="F111">
+        <v>30</v>
+      </c>
+      <c r="G111" t="s">
+        <v>8</v>
+      </c>
+      <c r="H111">
+        <v>1</v>
+      </c>
+      <c r="I111">
+        <v>119</v>
+      </c>
+      <c r="J111">
+        <v>119</v>
+      </c>
+      <c r="K111">
         <v>98</v>
       </c>
-      <c r="F111">
-        <v>28</v>
-      </c>
-      <c r="K111">
-        <v>43</v>
-      </c>
       <c r="L111">
-        <v>98</v>
+        <v>119</v>
       </c>
     </row>
     <row r="112" spans="1:12" x14ac:dyDescent="0.25">
@@ -3342,37 +3378,25 @@
         <v>43</v>
       </c>
       <c r="B112">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C112" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D112" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E112">
-        <v>39</v>
+        <v>95</v>
       </c>
       <c r="F112">
-        <v>39</v>
-      </c>
-      <c r="G112" t="s">
-        <v>8</v>
-      </c>
-      <c r="H112">
-        <v>1</v>
-      </c>
-      <c r="I112">
-        <v>119</v>
-      </c>
-      <c r="J112">
-        <v>119</v>
+        <v>30</v>
       </c>
       <c r="K112">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="L112">
-        <v>119</v>
+        <v>95</v>
       </c>
     </row>
     <row r="113" spans="1:12" x14ac:dyDescent="0.25">
@@ -3380,34 +3404,34 @@
         <v>43</v>
       </c>
       <c r="B113">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C113" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D113" t="s">
         <v>11</v>
       </c>
       <c r="E113">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="F113">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="G113" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H113">
         <v>1</v>
       </c>
       <c r="I113">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="J113">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="K113">
-        <v>65</v>
+        <v>105</v>
       </c>
       <c r="L113">
         <v>119</v>
@@ -3418,19 +3442,37 @@
         <v>43</v>
       </c>
       <c r="B114">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C114" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D114" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E114">
-        <v>77</v>
+        <v>35</v>
+      </c>
+      <c r="F114">
+        <v>35</v>
+      </c>
+      <c r="G114" t="s">
+        <v>25</v>
+      </c>
+      <c r="H114">
+        <v>0</v>
+      </c>
+      <c r="I114">
+        <v>95</v>
+      </c>
+      <c r="J114">
+        <v>95</v>
+      </c>
+      <c r="K114">
+        <v>65</v>
       </c>
       <c r="L114">
-        <v>77</v>
+        <v>119</v>
       </c>
     </row>
     <row r="115" spans="1:12" x14ac:dyDescent="0.25">
@@ -3438,17 +3480,23 @@
         <v>43</v>
       </c>
       <c r="B115">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C115" t="s">
         <v>3</v>
       </c>
       <c r="D115" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E115">
         <v>98</v>
       </c>
+      <c r="F115">
+        <v>28</v>
+      </c>
+      <c r="K115">
+        <v>43</v>
+      </c>
       <c r="L115">
         <v>98</v>
       </c>
@@ -3458,19 +3506,37 @@
         <v>43</v>
       </c>
       <c r="B116">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="C116" t="s">
         <v>3</v>
       </c>
       <c r="D116" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E116">
-        <v>77</v>
+        <v>39</v>
+      </c>
+      <c r="F116">
+        <v>39</v>
+      </c>
+      <c r="G116" t="s">
+        <v>8</v>
+      </c>
+      <c r="H116">
+        <v>1</v>
+      </c>
+      <c r="I116">
+        <v>119</v>
+      </c>
+      <c r="J116">
+        <v>119</v>
+      </c>
+      <c r="K116">
+        <v>65</v>
       </c>
       <c r="L116">
-        <v>77</v>
+        <v>119</v>
       </c>
     </row>
     <row r="117" spans="1:12" x14ac:dyDescent="0.25">
@@ -3478,19 +3544,37 @@
         <v>43</v>
       </c>
       <c r="B117">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="C117" t="s">
         <v>3</v>
       </c>
       <c r="D117" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E117">
-        <v>77</v>
+        <v>49</v>
+      </c>
+      <c r="F117">
+        <v>49</v>
+      </c>
+      <c r="G117" t="s">
+        <v>13</v>
+      </c>
+      <c r="H117">
+        <v>1</v>
+      </c>
+      <c r="I117">
+        <v>119</v>
+      </c>
+      <c r="J117">
+        <v>112</v>
+      </c>
+      <c r="K117">
+        <v>65</v>
       </c>
       <c r="L117">
-        <v>77</v>
+        <v>119</v>
       </c>
     </row>
     <row r="118" spans="1:12" x14ac:dyDescent="0.25">
@@ -3498,7 +3582,7 @@
         <v>43</v>
       </c>
       <c r="B118">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="C118" t="s">
         <v>3</v>
@@ -3507,10 +3591,10 @@
         <v>8</v>
       </c>
       <c r="E118">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="L118">
-        <v>98</v>
+        <v>77</v>
       </c>
     </row>
     <row r="119" spans="1:12" x14ac:dyDescent="0.25">
@@ -3518,25 +3602,19 @@
         <v>43</v>
       </c>
       <c r="B119">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="C119" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D119" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E119">
-        <v>95</v>
-      </c>
-      <c r="F119">
-        <v>14</v>
-      </c>
-      <c r="K119">
-        <v>58</v>
+        <v>98</v>
       </c>
       <c r="L119">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="120" spans="1:12" x14ac:dyDescent="0.25">
@@ -3544,19 +3622,37 @@
         <v>43</v>
       </c>
       <c r="B120">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="C120" t="s">
         <v>4</v>
       </c>
       <c r="D120" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E120">
-        <v>77</v>
+        <v>119</v>
+      </c>
+      <c r="F120">
+        <v>43</v>
+      </c>
+      <c r="G120" t="s">
+        <v>13</v>
+      </c>
+      <c r="H120">
+        <v>1</v>
+      </c>
+      <c r="I120">
+        <v>119</v>
+      </c>
+      <c r="J120">
+        <v>109</v>
+      </c>
+      <c r="K120">
+        <v>87</v>
       </c>
       <c r="L120">
-        <v>77</v>
+        <v>119</v>
       </c>
     </row>
     <row r="121" spans="1:12" x14ac:dyDescent="0.25">
@@ -3564,34 +3660,34 @@
         <v>43</v>
       </c>
       <c r="B121">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="C121" t="s">
         <v>4</v>
       </c>
       <c r="D121" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E121">
-        <v>35</v>
+        <v>119</v>
       </c>
       <c r="F121">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G121" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H121">
         <v>1</v>
       </c>
       <c r="I121">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="J121">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="K121">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="L121">
         <v>119</v>
@@ -3602,7 +3698,7 @@
         <v>43</v>
       </c>
       <c r="B122">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="C122" t="s">
         <v>4</v>
@@ -3611,28 +3707,16 @@
         <v>10</v>
       </c>
       <c r="E122">
-        <v>119</v>
+        <v>92</v>
       </c>
       <c r="F122">
         <v>30</v>
       </c>
-      <c r="G122" t="s">
-        <v>8</v>
-      </c>
-      <c r="H122">
-        <v>1</v>
-      </c>
-      <c r="I122">
-        <v>119</v>
-      </c>
-      <c r="J122">
-        <v>119</v>
-      </c>
       <c r="K122">
-        <v>98</v>
+        <v>39</v>
       </c>
       <c r="L122">
-        <v>119</v>
+        <v>92</v>
       </c>
     </row>
     <row r="123" spans="1:12" x14ac:dyDescent="0.25">
@@ -3640,7 +3724,7 @@
         <v>43</v>
       </c>
       <c r="B123">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="C123" t="s">
         <v>4</v>
@@ -3649,16 +3733,28 @@
         <v>10</v>
       </c>
       <c r="E123">
-        <v>95</v>
+        <v>119</v>
       </c>
       <c r="F123">
         <v>30</v>
       </c>
+      <c r="G123" t="s">
+        <v>8</v>
+      </c>
+      <c r="H123">
+        <v>1</v>
+      </c>
+      <c r="I123">
+        <v>119</v>
+      </c>
+      <c r="J123">
+        <v>119</v>
+      </c>
       <c r="K123">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="L123">
-        <v>95</v>
+        <v>119</v>
       </c>
     </row>
     <row r="124" spans="1:12" x14ac:dyDescent="0.25">
@@ -3666,37 +3762,19 @@
         <v>43</v>
       </c>
       <c r="B124">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="C124" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="D124" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E124">
-        <v>30</v>
-      </c>
-      <c r="F124">
-        <v>30</v>
-      </c>
-      <c r="G124" t="s">
-        <v>12</v>
-      </c>
-      <c r="H124">
-        <v>1</v>
-      </c>
-      <c r="I124">
-        <v>105</v>
-      </c>
-      <c r="J124">
-        <v>105</v>
-      </c>
-      <c r="K124">
-        <v>105</v>
+        <v>77</v>
       </c>
       <c r="L124">
-        <v>119</v>
+        <v>77</v>
       </c>
     </row>
     <row r="125" spans="1:12" x14ac:dyDescent="0.25">
@@ -3704,37 +3782,19 @@
         <v>43</v>
       </c>
       <c r="B125">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="C125" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="D125" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E125">
-        <v>35</v>
-      </c>
-      <c r="F125">
-        <v>35</v>
-      </c>
-      <c r="G125" t="s">
-        <v>25</v>
-      </c>
-      <c r="H125">
-        <v>0</v>
-      </c>
-      <c r="I125">
-        <v>95</v>
-      </c>
-      <c r="J125">
-        <v>95</v>
-      </c>
-      <c r="K125">
-        <v>65</v>
+        <v>77</v>
       </c>
       <c r="L125">
-        <v>119</v>
+        <v>77</v>
       </c>
     </row>
     <row r="126" spans="1:12" x14ac:dyDescent="0.25">
@@ -3742,37 +3802,19 @@
         <v>43</v>
       </c>
       <c r="B126">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="C126" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="D126" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E126">
-        <v>119</v>
-      </c>
-      <c r="F126">
-        <v>43</v>
-      </c>
-      <c r="G126" t="s">
-        <v>13</v>
-      </c>
-      <c r="H126">
-        <v>1</v>
-      </c>
-      <c r="I126">
-        <v>119</v>
-      </c>
-      <c r="J126">
-        <v>109</v>
-      </c>
-      <c r="K126">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="L126">
-        <v>119</v>
+        <v>72</v>
       </c>
     </row>
     <row r="127" spans="1:12" x14ac:dyDescent="0.25">
@@ -3780,37 +3822,19 @@
         <v>43</v>
       </c>
       <c r="B127">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="C127" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D127" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E127">
-        <v>119</v>
-      </c>
-      <c r="F127">
-        <v>30</v>
-      </c>
-      <c r="G127" t="s">
-        <v>8</v>
-      </c>
-      <c r="H127">
-        <v>1</v>
-      </c>
-      <c r="I127">
-        <v>119</v>
-      </c>
-      <c r="J127">
-        <v>119</v>
-      </c>
-      <c r="K127">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="L127">
-        <v>119</v>
+        <v>77</v>
       </c>
     </row>
     <row r="128" spans="1:12" x14ac:dyDescent="0.25">
@@ -3818,25 +3842,19 @@
         <v>43</v>
       </c>
       <c r="B128">
-        <v>37</v>
+        <v>49</v>
       </c>
       <c r="C128" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D128" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E128">
-        <v>92</v>
-      </c>
-      <c r="F128">
-        <v>30</v>
-      </c>
-      <c r="K128">
-        <v>39</v>
+        <v>77</v>
       </c>
       <c r="L128">
-        <v>92</v>
+        <v>77</v>
       </c>
     </row>
     <row r="129" spans="1:12" x14ac:dyDescent="0.25">
@@ -3844,37 +3862,19 @@
         <v>43</v>
       </c>
       <c r="B129">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="C129" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D129" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E129">
-        <v>119</v>
-      </c>
-      <c r="F129">
-        <v>30</v>
-      </c>
-      <c r="G129" t="s">
-        <v>8</v>
-      </c>
-      <c r="H129">
-        <v>1</v>
-      </c>
-      <c r="I129">
-        <v>119</v>
-      </c>
-      <c r="J129">
-        <v>119</v>
-      </c>
-      <c r="K129">
-        <v>58</v>
+        <v>98</v>
       </c>
       <c r="L129">
-        <v>119</v>
+        <v>98</v>
       </c>
     </row>
     <row r="130" spans="1:12" x14ac:dyDescent="0.25">
@@ -4252,6 +4252,10 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L142">
+    <sortCondition ref="A2:A142"/>
+    <sortCondition ref="B2:B142"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>

</xml_diff>